<commit_message>
Size the 5 Whys example rows to their content
A fixed 30pt row clipped the last wrapped line of every branch, which is exactly
the line naming the root cause — "no one owned the ticket lifecycle when it was
designed" rendered as "when it was". Rows are now sized from their longest cell.
</commit_message>
<xml_diff>
--- a/templates/20-five-whys-tree.xlsx
+++ b/templates/20-five-whys-tree.xlsx
@@ -814,7 +814,7 @@
         </is>
       </c>
     </row>
-    <row r="10" ht="30" customHeight="1">
+    <row r="10" ht="60" customHeight="1">
       <c r="A10" s="11" t="inlineStr">
         <is>
           <t>1</t>
@@ -861,7 +861,7 @@
         </is>
       </c>
     </row>
-    <row r="11" ht="30" customHeight="1">
+    <row r="11" ht="45" customHeight="1">
       <c r="A11" s="11" t="inlineStr">
         <is>
           <t>2</t>
@@ -908,7 +908,7 @@
         </is>
       </c>
     </row>
-    <row r="12" ht="30" customHeight="1">
+    <row r="12" ht="45" customHeight="1">
       <c r="A12" s="11" t="inlineStr">
         <is>
           <t>3</t>

</xml_diff>